<commit_message>
Rows&Columns 1.1: version 1.1.0, version log and decisions D12-D15
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/VERSION_LOG.xlsx
+++ b/VERSION_LOG.xlsx
@@ -11,7 +11,7 @@
     <sheet name="How versions work" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Versions'!$A$1:$I$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Versions'!$A$1:$I$3</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -549,8 +549,58 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Big sheets load completely; Excel-like dark theme</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>• Big XLSX sheets now load completely. Sheets with more than ~1,000,000 cells were reported 'damaged' and only the first ~71,000 rows loaded, so saving would have lost rows (G09; upstream #2526 still open). 300,001-row test file: 1.0 kept 71,428 rows, 1.1 loads all.
+• Dark theme colours measured from Excel for Mac: near-black frame, lighter ribbon, near-black headings with white letters, light-green band with dark-green letters for a fully selected column or row, grey selection tint, darker dialogs and menus, green list selection (G05, colours part).
+• Includes 55 newer GridCraft commits (upstream main 45f5ab18, 2026-10-27); our earlier fixes re-applied in their reorganised files.
+• Official GridCraft app removed from Applications at the owner's request; pushing to GridCraft's repository is blocked locally.</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>G09, G05 (colours)</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>0.12.1 + main 45f5ab18</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>v1.1.0</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Released</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I2"/>
+  <autoFilter ref="A1:I3"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Rows&Columns 1.2: version 1.2.0, version log, decisions D16-D17, README
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/VERSION_LOG.xlsx
+++ b/VERSION_LOG.xlsx
@@ -11,7 +11,7 @@
     <sheet name="How versions work" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Versions'!$A$1:$I$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Versions'!$A$1:$I$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -599,8 +599,58 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Excel-style filter menu: Auto Apply, conditions, date tree</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>• New filter dropdown laid out like Excel's (G06): the column's name as its title, Ascending / Descending side by side, 'Choose One' conditions that suit the column (text: equals, begins with, ends with, contains…; numbers: greater/less than, between, Top 10, above/below average; dates: before, after, between), search, Auto Apply (on by default: a tick filters straight away; off: changes wait for Apply Filter), Apply Filter and Clear Filter.
+• Date columns list as Year › Month › Day (newest year first) with expand arrows and part-ticked groups, like Excel (G12).
+• Big columns open fast: the value list is read once when the menu opens and drawn a screenful at a time (it was rebuilt on every screen refresh). One filter change on 300,000 rows: ~50 ms.
+• Includes 32 newer GridCraft commits (faster XLSX saving and fixes; upstream main 146161b4).</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>G06 (except filter/sort by colour), G12</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>0.13.0 + main 146161b4</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>v1.2.0</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>Released</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I3"/>
+  <autoFilter ref="A1:I4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Rows&Columns 1.3: version 1.3.0, version log, decision D18, README
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/VERSION_LOG.xlsx
+++ b/VERSION_LOG.xlsx
@@ -11,7 +11,7 @@
     <sheet name="How versions work" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Versions'!$A$1:$I$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Versions'!$A$1:$I$5</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -649,8 +649,58 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>1.3</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Day-month-year dates: Text to Columns and CSV opening</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>• Text to Columns gets Excel's 'Column data format': General, Text, Date in an order (DMY, MDY, YMD, MYD, DYM, YDM) or Skip. Date: DMY re-reads a column of day-month-year dates, including ones already turned into the wrong date (7/8/2024 → 7 August) and ones left as text (16-08-2023 → 16 August) (G02).
+• Opening a CSV: a column whose dates are clearly day first (some have a day over 12, none a month over 12) is read day first, so these files open correctly without Text to Columns. Better than Excel, which reads them month first. Unclear or mixed columns read as before (G02).
+• Impossible dates (month 16, 31 February) are left as written instead of rolling over.
+• CSV opening does one extra quick pass: about 0.1 s per 12 MB.</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>G02</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>0.13.0 + main 146161b4</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>v1.3.0</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>Released</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I4"/>
+  <autoFilter ref="A1:I5"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Rows&Columns 1.4: version 1.4.0, version log, decision D19, README
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/VERSION_LOG.xlsx
+++ b/VERSION_LOG.xlsx
@@ -11,7 +11,7 @@
     <sheet name="How versions work" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Versions'!$A$1:$I$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Versions'!$A$1:$I$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -699,8 +699,57 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Big files open without freezing; Remove Duplicates 3× faster</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>• Files of 2 MB or more open on a background thread: the window stays responsive and shows 'Opening &lt;file&gt;… N s · Esc to cancel' instead of a spinning beach ball. Esc cancels. Smaller files open instantly as before (G07, part 1).
+• Remove Duplicates on 350,000 rows × 12 columns: ~7 s → ~2 s. Any command that changes millions of cells (big pastes, sorts, clears) no longer scans a 64×64 block around every changed cell (G07).
+• Still to do for G07: saving big files in the background, and progress with Esc for other long commands.</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>G07 (part)</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>0.13.0 + main 146161b4</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>v1.4.0</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>Released</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I5"/>
+  <autoFilter ref="A1:I6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Rows&Columns 1.5: version 1.5.0, version log, decision D20, README
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/VERSION_LOG.xlsx
+++ b/VERSION_LOG.xlsx
@@ -11,7 +11,7 @@
     <sheet name="How versions work" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Versions'!$A$1:$I$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Versions'!$A$1:$I$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -748,8 +748,58 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>1.5</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Excel-style checkboxes and buttons</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>• Every checkbox (dialogs, filter menu, Backstage, ribbon, panes; 44 in all) looks like Excel's: a rounded box that fills green with a white tick when on, and a white dash when part-ticked (G05).
+• Dialogs' main buttons (OK, Solve) are Excel's darker green with white text (G05).
+• The filter menu's date tree uses small grey chevrons instead of large triangles.
+• Still to do for G05: the icon set (style to be chosen with the owner).</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>G05 (dialogs &amp; widgets)</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>0.13.0 + main 146161b4</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>v1.5.0</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>Released</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I6"/>
+  <autoFilter ref="A1:I7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Rows&Columns 1.6: version 1.6.0, version log, decision D21, README
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/VERSION_LOG.xlsx
+++ b/VERSION_LOG.xlsx
@@ -11,7 +11,7 @@
     <sheet name="How versions work" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Versions'!$A$1:$I$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Versions'!$A$1:$I$8</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:I8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -798,8 +798,57 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Livelier icons; GridCraft macro recorder</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>• Ribbon icons redrawn with filled colour instead of thin outlines: Filter, Find, Sort &amp; Filter, Comment, Data Validation, Freeze Panes, Text to Columns, Remove Duplicates, Table and PivotTable. Every icon also gets subtle depth (a darker lower half and edge on coloured shapes) and slightly bolder lines (G05).
+• Includes 232 newer GridCraft commits: a macro recorder and step-by-step macro editor (Automate › Macros) plus engine fixes. Their new screens use Rows&amp;Columns' name and Excel-style checkboxes.
+• Dark-mode breakpoint dot lightened to stay readable on the green current-step highlight.</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>G05 (icons, first pass)</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>0.13.0 + main 2ff75179</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>v1.6.0</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>Released</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I7"/>
+  <autoFilter ref="A1:I8"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Rows&Columns 1.7: version 1.7.0, version log, decisions D22-D23, README
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/VERSION_LOG.xlsx
+++ b/VERSION_LOG.xlsx
@@ -11,7 +11,7 @@
     <sheet name="How versions work" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Versions'!$A$1:$I$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Versions'!$A$1:$I$9</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -847,8 +847,56 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>1.7</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Big files save in the background; Excel's narrow font fits numbers</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>• Saving a big workbook (200,000+ cells) with ⌘S or File › Save happens in the background with 'Saving &lt;file&gt;… N s' in the corner; the window stays usable. Edits made during the save stay marked unsaved. Quitting during a save waits for it, then quits as usual. Saves from the quit prompt and from scripts stay immediate (G07).
+• Workbooks in Excel's default font, Aptos Narrow, now draw with a narrow font when Aptos isn't installed (Arial Narrow on a Mac), so numbers fit their columns as in Excel: 2403607 instead of 2E+06 (G11).</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>G07, G11</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>0.13.0 + main 2ff75179</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>v1.7.0</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>Released</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I8"/>
+  <autoFilter ref="A1:I9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Rows&Columns 1.8: version 1.8.0, version log, README
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/VERSION_LOG.xlsx
+++ b/VERSION_LOG.xlsx
@@ -11,7 +11,7 @@
     <sheet name="How versions work" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Versions'!$A$1:$I$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Versions'!$A$1:$I$10</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -895,8 +895,55 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>1.8</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Excel pivots with date grouping open cleanly</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>• PivotTables made in Excel with automatic date grouping (Years › Quarters › Months › dates) open without the 'grouping is not supported' warning; the levels and collapsed years are kept as in Excel (G10). Checked on the owner's acquisitions pivot file.</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>G10</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>0.13.0 + main 2ff75179</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>v1.8.0</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>Released</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I9"/>
+  <autoFilter ref="A1:I10"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Rows&Columns 1.9: version 1.9.0, version log, README
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/VERSION_LOG.xlsx
+++ b/VERSION_LOG.xlsx
@@ -11,7 +11,7 @@
     <sheet name="How versions work" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Versions'!$A$1:$I$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Versions'!$A$1:$I$11</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -942,8 +942,51 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>1.9</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>New app icon (temporary)</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>• Rows&amp;Columns has its own app icon: a green glass spreadsheet tile provided by the owner, used in Finder, Launchpad and the Dock. Temporary: a final icon will replace it later.</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr"/>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>0.13.0 + main 2ff75179</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>v1.9.0</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>Released</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I10"/>
+  <autoFilter ref="A1:I11"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>